<commit_message>
Fix pricing import and basis review flows
</commit_message>
<xml_diff>
--- a/pricing-references/_template/swooshz-pricing-reference-template.xlsx
+++ b/pricing-references/_template/swooshz-pricing-reference-template.xlsx
@@ -10,7 +10,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:G9"/>
   <cols>
     <col min="1" max="1" width="0" hidden="1" customWidth="1"/>
     <col min="2" max="2" width="24" customWidth="1"/>
@@ -18,7 +18,6 @@
     <col min="4" max="4" width="14" customWidth="1"/>
     <col min="5" max="6" width="18" customWidth="1"/>
     <col min="7" max="7" width="36" customWidth="1"/>
-    <col min="8" max="8" width="56" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -57,11 +56,6 @@
           <t>remarks</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>aliases</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -99,11 +93,6 @@
           <t>needle punch</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>needle punch carpet in colour|needle punch|carpet sqm</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -141,11 +130,6 @@
           <t>Platform ONLY</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>raised platform|platform|aluminum edging</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -183,11 +167,6 @@
           <t>Backwall or any partition; PAINTED</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>partition wall|painted backwall|wooden partition</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -225,11 +204,6 @@
           <t>INFORMATION COUNTER; PAINTED</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>information counter|lockable counter|counter laminated top</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -267,11 +241,6 @@
           <t>SPOTLIGHT</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>spotlight|LED light|10W light</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -309,11 +278,6 @@
           <t>Printed Graphics on wall</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>vinyl graphics|printed graphics|wall graphics</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -351,11 +315,6 @@
           <t>Bistro Low Chair</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>bistro chairs|low chair|chair rental</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -391,11 +350,6 @@
       <c r="G9" t="inlineStr">
         <is>
           <t>TV</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>LED TV|screen|monitor|42 inch TV</t>
         </is>
       </c>
     </row>
@@ -405,7 +359,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B9"/>
   <cols>
     <col min="1" max="1" width="72" customWidth="1"/>
     <col min="2" max="2" width="72" customWidth="1"/>
@@ -505,19 +459,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Optional. Internal matching/search notes; separate multiple values with semicolon.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>aliases</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Optional. Separate search aliases with | or ;.</t>
+          <t>Optional. Internal matching/search notes; separate multiple values with semicolon. AI-generated aliases are added during import.</t>
         </is>
       </c>
     </row>

</xml_diff>